<commit_message>
Update tracker, site zip, settings, and business card PDF
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cameroon_Shop_Purchase_Tracker.xlsx
+++ b/Cameroon_Shop_Purchase_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\cameroon-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB16E567-6397-4C72-ACD9-032472C1A096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42CF9A79-B8ED-4FA2-8370-C19FB7EACCAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-2616" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="141">
   <si>
     <t>TOTAL PURCHASE COST</t>
   </si>
@@ -436,6 +436,27 @@
   </si>
   <si>
     <t>Dr Teals Body Wash/Lotion</t>
+  </si>
+  <si>
+    <t>Fabreze Air Freshener</t>
+  </si>
+  <si>
+    <t>4 (2)</t>
+  </si>
+  <si>
+    <t>Crest Mouth Wash</t>
+  </si>
+  <si>
+    <t>9 (3)</t>
+  </si>
+  <si>
+    <t>Irish Springs</t>
+  </si>
+  <si>
+    <t>Degree Deodorant</t>
+  </si>
+  <si>
+    <t>10(5)</t>
   </si>
 </sst>
 </file>
@@ -542,7 +563,12 @@
       <family val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF2C3E50"/>
       <name val="Times New Roman"/>
@@ -550,18 +576,12 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF222222"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <color rgb="FF0F1111"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF0F1111"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="14"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -673,21 +693,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="8" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="8" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="6" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="8" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="8" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="8" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -697,28 +702,43 @@
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="8" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="6" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="8" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="6" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="15" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="18" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1021,17 +1041,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.140625" customWidth="1"/>
-    <col min="2" max="2" width="23.42578125" style="40" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" style="31" customWidth="1"/>
     <col min="3" max="3" width="25.85546875" customWidth="1"/>
     <col min="4" max="4" width="22.42578125" style="2" customWidth="1"/>
     <col min="5" max="5" width="11.42578125" style="28" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" style="22" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.28515625" customWidth="1"/>
-    <col min="8" max="8" width="24.85546875" style="31" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" style="39" customWidth="1"/>
     <col min="9" max="9" width="18.42578125" customWidth="1"/>
     <col min="10" max="10" width="25" customWidth="1"/>
   </cols>
@@ -1040,9 +1060,9 @@
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40">
+      <c r="B1" s="31">
         <f>SUM(F:F)</f>
-        <v>452.55</v>
+        <v>303.89999999999998</v>
       </c>
       <c r="C1" s="8"/>
       <c r="D1" s="9"/>
@@ -1058,7 +1078,7 @@
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40">
+      <c r="B2" s="31">
         <f>SUM(G:G)</f>
         <v>77.8</v>
       </c>
@@ -1076,9 +1096,9 @@
       <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="40">
+      <c r="B3" s="31">
         <f>SUM(H:H)</f>
-        <v>2088.3199999999997</v>
+        <v>2386.9499999999998</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="9"/>
@@ -1094,7 +1114,7 @@
       <c r="A4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="40">
+      <c r="B4" s="31">
         <f>SUM(K:K)</f>
         <v>0</v>
       </c>
@@ -1124,7 +1144,7 @@
       <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -1142,7 +1162,7 @@
       <c r="G6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="31" t="s">
+      <c r="H6" s="39" t="s">
         <v>11</v>
       </c>
       <c r="I6" s="8" t="s">
@@ -1162,7 +1182,7 @@
       <c r="A7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="32" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="8"/>
@@ -1189,7 +1209,7 @@
     </row>
     <row r="8" spans="1:12" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A8" s="8"/>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="32" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="8"/>
@@ -1208,7 +1228,7 @@
     </row>
     <row r="9" spans="1:12" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A9" s="8"/>
-      <c r="B9" s="41" t="s">
+      <c r="B9" s="32" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="8"/>
@@ -1227,7 +1247,7 @@
     </row>
     <row r="10" spans="1:12" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="32" t="s">
         <v>20</v>
       </c>
       <c r="C10" s="8"/>
@@ -1246,7 +1266,7 @@
     </row>
     <row r="11" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A11" s="8"/>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="32" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="8"/>
@@ -1265,7 +1285,7 @@
     </row>
     <row r="12" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="32" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="8"/>
@@ -1284,7 +1304,7 @@
     </row>
     <row r="13" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A13" s="8"/>
-      <c r="B13" s="41" t="s">
+      <c r="B13" s="32" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="8"/>
@@ -1303,7 +1323,7 @@
     </row>
     <row r="14" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A14" s="8"/>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="32" t="s">
         <v>24</v>
       </c>
       <c r="C14" s="8"/>
@@ -1322,7 +1342,7 @@
     </row>
     <row r="15" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="32" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="8"/>
@@ -1341,7 +1361,7 @@
     </row>
     <row r="16" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A16" s="8"/>
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="32" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="8"/>
@@ -1360,7 +1380,7 @@
     </row>
     <row r="17" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A17" s="8"/>
-      <c r="B17" s="41" t="s">
+      <c r="B17" s="32" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="8"/>
@@ -1379,7 +1399,7 @@
     </row>
     <row r="18" spans="1:12" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A18" s="8"/>
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="32" t="s">
         <v>28</v>
       </c>
       <c r="C18" s="8"/>
@@ -1398,7 +1418,7 @@
     </row>
     <row r="19" spans="1:12" s="13" customFormat="1" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A19" s="16"/>
-      <c r="B19" s="40"/>
+      <c r="B19" s="31"/>
       <c r="C19" s="16"/>
       <c r="D19" s="17"/>
       <c r="E19" s="27"/>
@@ -1406,7 +1426,7 @@
       <c r="G19" s="18">
         <v>23.94</v>
       </c>
-      <c r="H19" s="48">
+      <c r="H19" s="40">
         <v>104.79</v>
       </c>
       <c r="I19" s="16"/>
@@ -1415,7 +1435,7 @@
       <c r="L19" s="16"/>
     </row>
     <row r="20" spans="1:12" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="32" t="s">
         <v>30</v>
       </c>
       <c r="D20" s="3" t="s">
@@ -1430,7 +1450,7 @@
       <c r="G20" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="H20" s="48">
+      <c r="H20" s="40">
         <v>69.73</v>
       </c>
     </row>
@@ -1447,13 +1467,13 @@
       <c r="G21" s="4">
         <v>32.799999999999997</v>
       </c>
-      <c r="H21" s="35"/>
+      <c r="H21" s="41"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
         <v>46050</v>
       </c>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="31" t="s">
         <v>31</v>
       </c>
       <c r="D22" s="3"/>
@@ -1465,7 +1485,7 @@
       <c r="A24" s="5">
         <v>46053</v>
       </c>
-      <c r="B24" s="40" t="s">
+      <c r="B24" s="31" t="s">
         <v>33</v>
       </c>
       <c r="C24" t="s">
@@ -1483,7 +1503,7 @@
       <c r="G24">
         <v>7.92</v>
       </c>
-      <c r="H24" s="32">
+      <c r="H24" s="42">
         <v>62.81</v>
       </c>
     </row>
@@ -1491,7 +1511,7 @@
       <c r="A25" s="5">
         <v>46053</v>
       </c>
-      <c r="B25" s="40" t="s">
+      <c r="B25" s="31" t="s">
         <v>35</v>
       </c>
       <c r="C25" t="s">
@@ -1509,12 +1529,12 @@
       <c r="G25" s="4">
         <v>13.14</v>
       </c>
-      <c r="H25" s="32">
+      <c r="H25" s="42">
         <v>53.14</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="40" t="s">
+      <c r="B26" s="31" t="s">
         <v>37</v>
       </c>
       <c r="C26" t="s">
@@ -1529,12 +1549,12 @@
       <c r="F26" s="23">
         <v>8</v>
       </c>
-      <c r="H26" s="32">
+      <c r="H26" s="42">
         <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="40" t="s">
+      <c r="B27" s="31" t="s">
         <v>41</v>
       </c>
       <c r="C27" t="s">
@@ -1549,12 +1569,12 @@
       <c r="F27" s="22">
         <v>8</v>
       </c>
-      <c r="H27" s="32">
+      <c r="H27" s="42">
         <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B28" s="42" t="s">
+      <c r="B28" s="33" t="s">
         <v>43</v>
       </c>
       <c r="D28" s="2" t="s">
@@ -1566,12 +1586,12 @@
       <c r="F28" s="22">
         <v>10</v>
       </c>
-      <c r="H28" s="32">
+      <c r="H28" s="42">
         <v>34.89</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B29" s="42" t="s">
+      <c r="B29" s="33" t="s">
         <v>45</v>
       </c>
       <c r="D29" s="2" t="s">
@@ -1583,12 +1603,12 @@
       <c r="F29" s="22">
         <v>10</v>
       </c>
-      <c r="H29" s="33">
+      <c r="H29" s="43">
         <v>34.86</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B30" s="42" t="s">
+      <c r="B30" s="33" t="s">
         <v>46</v>
       </c>
       <c r="D30" s="2" t="s">
@@ -1597,12 +1617,12 @@
       <c r="E30" s="28">
         <v>3</v>
       </c>
-      <c r="H30" s="33">
+      <c r="H30" s="43">
         <v>45.07</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="27" x14ac:dyDescent="0.3">
-      <c r="B31" s="42" t="s">
+      <c r="B31" s="33" t="s">
         <v>47</v>
       </c>
       <c r="D31" s="2" t="s">
@@ -1611,12 +1631,12 @@
       <c r="E31" s="28">
         <v>3</v>
       </c>
-      <c r="H31" s="33">
+      <c r="H31" s="43">
         <v>51.26</v>
       </c>
     </row>
     <row r="32" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="42" t="s">
+      <c r="B32" s="33" t="s">
         <v>48</v>
       </c>
       <c r="D32" s="7" t="s">
@@ -1626,12 +1646,12 @@
         <v>1</v>
       </c>
       <c r="F32" s="22"/>
-      <c r="H32" s="33">
+      <c r="H32" s="43">
         <v>5.41</v>
       </c>
     </row>
     <row r="33" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B33" s="42" t="s">
+      <c r="B33" s="33" t="s">
         <v>49</v>
       </c>
       <c r="D33" s="7" t="s">
@@ -1640,12 +1660,12 @@
       <c r="E33" s="28">
         <v>3</v>
       </c>
-      <c r="H33" s="33">
+      <c r="H33" s="43">
         <v>27</v>
       </c>
     </row>
     <row r="34" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B34" s="42" t="s">
+      <c r="B34" s="33" t="s">
         <v>50</v>
       </c>
       <c r="D34" s="7" t="s">
@@ -1654,12 +1674,12 @@
       <c r="E34" s="28">
         <v>2</v>
       </c>
-      <c r="H34" s="33">
+      <c r="H34" s="43">
         <v>13.04</v>
       </c>
     </row>
     <row r="35" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B35" s="42" t="s">
+      <c r="B35" s="33" t="s">
         <v>51</v>
       </c>
       <c r="D35" s="7" t="s">
@@ -1668,12 +1688,12 @@
       <c r="E35" s="28">
         <v>2</v>
       </c>
-      <c r="H35" s="33">
+      <c r="H35" s="43">
         <v>25</v>
       </c>
     </row>
     <row r="36" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B36" s="42" t="s">
+      <c r="B36" s="33" t="s">
         <v>52</v>
       </c>
       <c r="D36" s="7" t="s">
@@ -1682,12 +1702,12 @@
       <c r="E36" s="28">
         <v>2</v>
       </c>
-      <c r="H36" s="33">
+      <c r="H36" s="43">
         <v>23</v>
       </c>
     </row>
     <row r="37" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B37" s="42" t="s">
+      <c r="B37" s="33" t="s">
         <v>53</v>
       </c>
       <c r="D37" s="7" t="s">
@@ -1696,12 +1716,12 @@
       <c r="E37" s="28">
         <v>1</v>
       </c>
-      <c r="H37" s="33">
+      <c r="H37" s="43">
         <v>5</v>
       </c>
     </row>
     <row r="38" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B38" s="42" t="s">
+      <c r="B38" s="33" t="s">
         <v>54</v>
       </c>
       <c r="D38" s="7" t="s">
@@ -1710,12 +1730,12 @@
       <c r="E38" s="28">
         <v>10</v>
       </c>
-      <c r="H38" s="33">
+      <c r="H38" s="43">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B39" s="42" t="s">
+      <c r="B39" s="33" t="s">
         <v>55</v>
       </c>
       <c r="D39" s="7" t="s">
@@ -1724,12 +1744,12 @@
       <c r="E39" s="28">
         <v>1</v>
       </c>
-      <c r="H39" s="33">
+      <c r="H39" s="43">
         <v>9</v>
       </c>
     </row>
     <row r="40" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B40" s="42" t="s">
+      <c r="B40" s="33" t="s">
         <v>56</v>
       </c>
       <c r="D40" s="7" t="s">
@@ -1738,12 +1758,12 @@
       <c r="E40" s="28">
         <v>1</v>
       </c>
-      <c r="H40" s="33">
+      <c r="H40" s="43">
         <v>3</v>
       </c>
     </row>
     <row r="41" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B41" s="42" t="s">
+      <c r="B41" s="33" t="s">
         <v>57</v>
       </c>
       <c r="D41" s="7" t="s">
@@ -1752,12 +1772,12 @@
       <c r="E41" s="28">
         <v>1</v>
       </c>
-      <c r="H41" s="33">
+      <c r="H41" s="43">
         <v>11</v>
       </c>
     </row>
     <row r="42" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B42" s="42" t="s">
+      <c r="B42" s="33" t="s">
         <v>58</v>
       </c>
       <c r="D42" s="7" t="s">
@@ -1766,12 +1786,12 @@
       <c r="E42" s="28">
         <v>1</v>
       </c>
-      <c r="H42" s="33">
+      <c r="H42" s="43">
         <v>12</v>
       </c>
     </row>
     <row r="43" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B43" s="42" t="s">
+      <c r="B43" s="33" t="s">
         <v>59</v>
       </c>
       <c r="D43" s="7" t="s">
@@ -1780,12 +1800,12 @@
       <c r="E43" s="28">
         <v>2</v>
       </c>
-      <c r="H43" s="33">
+      <c r="H43" s="43">
         <v>10</v>
       </c>
     </row>
     <row r="44" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B44" s="42" t="s">
+      <c r="B44" s="33" t="s">
         <v>60</v>
       </c>
       <c r="D44" s="7" t="s">
@@ -1794,12 +1814,12 @@
       <c r="E44" s="28">
         <v>5</v>
       </c>
-      <c r="H44" s="33">
+      <c r="H44" s="43">
         <v>5</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B45" s="42" t="s">
+      <c r="B45" s="33" t="s">
         <v>61</v>
       </c>
       <c r="D45" s="7" t="s">
@@ -1808,12 +1828,12 @@
       <c r="E45" s="28">
         <v>1</v>
       </c>
-      <c r="H45" s="33">
+      <c r="H45" s="43">
         <v>6</v>
       </c>
     </row>
     <row r="46" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B46" s="42" t="s">
+      <c r="B46" s="33" t="s">
         <v>62</v>
       </c>
       <c r="D46" s="7" t="s">
@@ -1822,12 +1842,12 @@
       <c r="E46" s="28">
         <v>2</v>
       </c>
-      <c r="H46" s="33">
+      <c r="H46" s="43">
         <v>22</v>
       </c>
     </row>
     <row r="47" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B47" s="42" t="s">
+      <c r="B47" s="33" t="s">
         <v>63</v>
       </c>
       <c r="D47" s="7" t="s">
@@ -1836,12 +1856,12 @@
       <c r="E47" s="28">
         <v>2</v>
       </c>
-      <c r="H47" s="33">
+      <c r="H47" s="43">
         <v>22</v>
       </c>
     </row>
     <row r="48" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B48" s="42" t="s">
+      <c r="B48" s="33" t="s">
         <v>64</v>
       </c>
       <c r="D48" s="7" t="s">
@@ -1850,12 +1870,12 @@
       <c r="E48" s="28">
         <v>1</v>
       </c>
-      <c r="H48" s="33">
+      <c r="H48" s="43">
         <v>12</v>
       </c>
     </row>
     <row r="49" spans="2:8" ht="89.25" x14ac:dyDescent="0.3">
-      <c r="B49" s="43" t="s">
+      <c r="B49" s="36" t="s">
         <v>65</v>
       </c>
       <c r="D49" s="7" t="s">
@@ -1864,12 +1884,12 @@
       <c r="E49" s="28">
         <v>1</v>
       </c>
-      <c r="H49" s="31">
+      <c r="H49" s="39">
         <v>5</v>
       </c>
     </row>
     <row r="50" spans="2:8" ht="38.25" x14ac:dyDescent="0.3">
-      <c r="B50" s="43" t="s">
+      <c r="B50" s="36" t="s">
         <v>66</v>
       </c>
       <c r="D50" s="7" t="s">
@@ -1878,12 +1898,12 @@
       <c r="E50" s="28">
         <v>1</v>
       </c>
-      <c r="H50" s="31">
+      <c r="H50" s="39">
         <v>5</v>
       </c>
     </row>
     <row r="52" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B52" s="41" t="s">
+      <c r="B52" s="32" t="s">
         <v>67</v>
       </c>
       <c r="D52" s="1" t="s">
@@ -1891,7 +1911,7 @@
       </c>
     </row>
     <row r="53" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B53" s="44" t="s">
+      <c r="B53" s="34" t="s">
         <v>68</v>
       </c>
       <c r="C53" s="11" t="s">
@@ -1904,12 +1924,12 @@
       <c r="F53" s="24">
         <v>5.95</v>
       </c>
-      <c r="H53" s="36" t="s">
+      <c r="H53" s="44" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="54" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B54" s="44" t="s">
+      <c r="B54" s="34" t="s">
         <v>71</v>
       </c>
       <c r="C54" s="11" t="s">
@@ -1922,12 +1942,12 @@
       <c r="F54" s="24">
         <v>5.95</v>
       </c>
-      <c r="H54" s="36" t="s">
+      <c r="H54" s="44" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="55" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B55" s="44" t="s">
+      <c r="B55" s="34" t="s">
         <v>73</v>
       </c>
       <c r="C55" s="11" t="s">
@@ -1940,12 +1960,12 @@
       <c r="F55" s="24">
         <v>5.95</v>
       </c>
-      <c r="H55" s="36" t="s">
+      <c r="H55" s="44" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="56" spans="2:8" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="B56" s="44" t="s">
+      <c r="B56" s="34" t="s">
         <v>75</v>
       </c>
       <c r="C56" s="11" t="s">
@@ -1958,12 +1978,12 @@
       <c r="F56" s="24">
         <v>5.95</v>
       </c>
-      <c r="H56" s="36" t="s">
+      <c r="H56" s="44" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="57" spans="2:8" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B57" s="44" t="s">
+      <c r="B57" s="34" t="s">
         <v>77</v>
       </c>
       <c r="C57" s="11" t="s">
@@ -1976,12 +1996,12 @@
       <c r="F57" s="24">
         <v>8.5</v>
       </c>
-      <c r="H57" s="36" t="s">
+      <c r="H57" s="44" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="58" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B58" s="44" t="s">
+      <c r="B58" s="34" t="s">
         <v>80</v>
       </c>
       <c r="C58" s="11" t="s">
@@ -1994,12 +2014,12 @@
       <c r="F58" s="24">
         <v>5.5</v>
       </c>
-      <c r="H58" s="36" t="s">
+      <c r="H58" s="44" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="59" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B59" s="44" t="s">
+      <c r="B59" s="34" t="s">
         <v>83</v>
       </c>
       <c r="C59" s="11" t="s">
@@ -2012,12 +2032,12 @@
       <c r="F59" s="24">
         <v>5.95</v>
       </c>
-      <c r="H59" s="36" t="s">
+      <c r="H59" s="44" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="60" spans="2:8" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B60" s="44" t="s">
+      <c r="B60" s="34" t="s">
         <v>85</v>
       </c>
       <c r="C60" s="11" t="s">
@@ -2030,12 +2050,12 @@
       <c r="F60" s="24">
         <v>5.5</v>
       </c>
-      <c r="H60" s="36" t="s">
+      <c r="H60" s="44" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="61" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B61" s="44" t="s">
+      <c r="B61" s="34" t="s">
         <v>87</v>
       </c>
       <c r="C61" s="11" t="s">
@@ -2048,12 +2068,12 @@
       <c r="F61" s="24">
         <v>5.5</v>
       </c>
-      <c r="H61" s="36" t="s">
+      <c r="H61" s="44" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="62" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B62" s="44" t="s">
+      <c r="B62" s="34" t="s">
         <v>89</v>
       </c>
       <c r="C62" s="11" t="s">
@@ -2066,24 +2086,24 @@
       <c r="F62" s="24">
         <v>5.75</v>
       </c>
-      <c r="H62" s="36" t="s">
+      <c r="H62" s="44" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="63" spans="2:8" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="40"/>
+      <c r="B63" s="31"/>
       <c r="D63" s="14"/>
       <c r="E63" s="28"/>
       <c r="F63" s="22"/>
       <c r="G63" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="H63" s="36" t="s">
+      <c r="H63" s="44" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="64" spans="2:8" ht="51.75" x14ac:dyDescent="0.25">
-      <c r="B64" s="45" t="s">
+      <c r="B64" s="35" t="s">
         <v>96</v>
       </c>
       <c r="E64" s="30">
@@ -2092,98 +2112,105 @@
       <c r="F64" s="25">
         <v>19.989999999999998</v>
       </c>
-      <c r="H64" s="35"/>
-    </row>
-    <row r="65" spans="2:11" ht="65.25" x14ac:dyDescent="0.3">
-      <c r="B65" s="45" t="s">
+      <c r="H64" s="41"/>
+    </row>
+    <row r="65" spans="2:11" ht="64.5" x14ac:dyDescent="0.25">
+      <c r="B65" s="35" t="s">
         <v>97</v>
       </c>
       <c r="E65" s="30">
         <v>3</v>
       </c>
-      <c r="F65" s="26">
+      <c r="F65" s="26"/>
+      <c r="H65" s="49">
         <v>14.17</v>
       </c>
     </row>
-    <row r="66" spans="2:11" ht="90.75" x14ac:dyDescent="0.3">
-      <c r="B66" s="45" t="s">
+    <row r="66" spans="2:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="B66" s="35" t="s">
         <v>98</v>
       </c>
       <c r="E66" s="30">
         <v>2</v>
       </c>
-      <c r="F66" s="26">
+      <c r="F66" s="26"/>
+      <c r="H66" s="49">
         <v>23.99</v>
       </c>
     </row>
-    <row r="67" spans="2:11" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B67" s="45" t="s">
+    <row r="67" spans="2:11" ht="51.75" x14ac:dyDescent="0.25">
+      <c r="B67" s="35" t="s">
         <v>99</v>
       </c>
       <c r="E67" s="30">
         <v>4</v>
       </c>
-      <c r="F67" s="26">
+      <c r="F67" s="26"/>
+      <c r="H67" s="49">
         <v>21.98</v>
       </c>
     </row>
-    <row r="68" spans="2:11" ht="78" x14ac:dyDescent="0.3">
-      <c r="B68" s="45" t="s">
+    <row r="68" spans="2:11" ht="77.25" x14ac:dyDescent="0.25">
+      <c r="B68" s="35" t="s">
         <v>100</v>
       </c>
       <c r="E68" s="30">
         <v>3</v>
       </c>
-      <c r="F68" s="26">
+      <c r="F68" s="26"/>
+      <c r="H68" s="49">
         <v>35.99</v>
       </c>
     </row>
-    <row r="69" spans="2:11" ht="78" x14ac:dyDescent="0.3">
-      <c r="B69" s="45" t="s">
+    <row r="69" spans="2:11" ht="77.25" x14ac:dyDescent="0.25">
+      <c r="B69" s="35" t="s">
         <v>101</v>
       </c>
       <c r="E69" s="30">
         <v>4</v>
       </c>
-      <c r="F69" s="26">
+      <c r="F69" s="26"/>
+      <c r="H69" s="49">
         <v>22.76</v>
       </c>
     </row>
-    <row r="70" spans="2:11" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B70" s="45" t="s">
+    <row r="70" spans="2:11" ht="51.75" x14ac:dyDescent="0.25">
+      <c r="B70" s="35" t="s">
         <v>102</v>
       </c>
       <c r="E70" s="30">
         <v>4</v>
       </c>
-      <c r="F70" s="26">
+      <c r="F70" s="26"/>
+      <c r="H70" s="49">
         <v>23.48</v>
       </c>
     </row>
-    <row r="71" spans="2:11" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B71" s="45" t="s">
+    <row r="71" spans="2:11" ht="51.75" x14ac:dyDescent="0.25">
+      <c r="B71" s="35" t="s">
         <v>106</v>
       </c>
       <c r="E71" s="30">
         <v>4</v>
       </c>
-      <c r="F71" s="26">
+      <c r="F71" s="26"/>
+      <c r="H71" s="49">
         <v>22.27</v>
       </c>
     </row>
-    <row r="72" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B72" s="46" t="s">
+    <row r="72" spans="2:11" ht="27" x14ac:dyDescent="0.3">
+      <c r="B72" s="37" t="s">
         <v>107</v>
       </c>
       <c r="E72" s="30">
         <v>6</v>
       </c>
-      <c r="H72" s="32">
+      <c r="H72" s="42">
         <v>38.26</v>
       </c>
     </row>
     <row r="73" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B73" s="46" t="s">
+      <c r="B73" s="37" t="s">
         <v>108</v>
       </c>
       <c r="E73" s="30">
@@ -2192,23 +2219,23 @@
       <c r="F73" s="23">
         <v>6</v>
       </c>
-      <c r="H73" s="32">
+      <c r="H73" s="42">
         <v>15.65</v>
       </c>
     </row>
-    <row r="74" spans="2:11" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B74" s="46" t="s">
+    <row r="74" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
+      <c r="B74" s="37" t="s">
         <v>109</v>
       </c>
       <c r="E74" s="30">
         <v>4</v>
       </c>
-      <c r="H74" s="32">
+      <c r="H74" s="42">
         <v>20.11</v>
       </c>
     </row>
     <row r="75" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B75" s="46" t="s">
+      <c r="B75" s="37" t="s">
         <v>110</v>
       </c>
       <c r="E75" s="30">
@@ -2216,40 +2243,40 @@
       </c>
     </row>
     <row r="76" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B76" s="46" t="s">
+      <c r="B76" s="37" t="s">
         <v>111</v>
       </c>
       <c r="E76" s="28">
         <v>15</v>
       </c>
-      <c r="H76" s="32">
+      <c r="H76" s="42">
         <v>31.5</v>
       </c>
     </row>
     <row r="77" spans="2:11" ht="27" x14ac:dyDescent="0.3">
-      <c r="B77" s="46" t="s">
+      <c r="B77" s="37" t="s">
         <v>130</v>
       </c>
       <c r="E77" s="28">
         <v>6</v>
       </c>
-      <c r="H77" s="32">
+      <c r="H77" s="42">
         <v>23</v>
       </c>
     </row>
     <row r="78" spans="2:11" ht="27" x14ac:dyDescent="0.3">
-      <c r="B78" s="46" t="s">
+      <c r="B78" s="37" t="s">
         <v>112</v>
       </c>
       <c r="E78" s="28">
         <v>1</v>
       </c>
-      <c r="H78" s="32">
+      <c r="H78" s="42">
         <v>10.34</v>
       </c>
     </row>
     <row r="79" spans="2:11" ht="27" x14ac:dyDescent="0.3">
-      <c r="B79" s="46" t="s">
+      <c r="B79" s="37" t="s">
         <v>113</v>
       </c>
       <c r="E79" s="28">
@@ -2258,21 +2285,21 @@
       <c r="F79" s="22">
         <v>3.68</v>
       </c>
-      <c r="H79" s="34">
+      <c r="H79" s="45">
         <v>23</v>
       </c>
     </row>
     <row r="80" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B80" s="46" t="s">
+      <c r="B80" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="H80" s="39">
+      <c r="H80" s="42">
         <v>16</v>
       </c>
       <c r="K80" s="13"/>
     </row>
-    <row r="81" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B81" s="46" t="s">
+    <row r="81" spans="2:8" ht="27" x14ac:dyDescent="0.3">
+      <c r="B81" s="37" t="s">
         <v>57</v>
       </c>
       <c r="E81" s="28">
@@ -2281,53 +2308,53 @@
       <c r="F81" s="22">
         <v>14</v>
       </c>
-      <c r="H81" s="34">
+      <c r="H81" s="45">
         <v>120</v>
       </c>
     </row>
-    <row r="82" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B82" s="46" t="s">
+    <row r="82" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
+      <c r="B82" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="H82" s="34">
+      <c r="H82" s="45">
         <v>75</v>
       </c>
     </row>
-    <row r="83" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B83" s="46" t="s">
+    <row r="83" spans="2:8" ht="27" x14ac:dyDescent="0.3">
+      <c r="B83" s="37" t="s">
         <v>116</v>
       </c>
       <c r="E83" s="28">
         <v>2</v>
       </c>
-      <c r="H83" s="34">
+      <c r="H83" s="45">
         <v>10</v>
       </c>
     </row>
-    <row r="84" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B84" s="46" t="s">
+    <row r="84" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
+      <c r="B84" s="37" t="s">
         <v>117</v>
       </c>
       <c r="E84" s="28">
         <v>4</v>
       </c>
-      <c r="H84" s="34">
+      <c r="H84" s="45">
         <v>40</v>
       </c>
     </row>
     <row r="85" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B85" s="46" t="s">
+      <c r="B85" s="37" t="s">
         <v>118</v>
       </c>
       <c r="E85" s="28">
         <v>20</v>
       </c>
-      <c r="H85" s="34">
+      <c r="H85" s="45">
         <v>90</v>
       </c>
     </row>
     <row r="86" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B86" s="46" t="s">
+      <c r="B86" s="37" t="s">
         <v>59</v>
       </c>
       <c r="E86" s="28">
@@ -2336,140 +2363,140 @@
       <c r="F86" s="22">
         <v>10.6</v>
       </c>
-      <c r="H86" s="37">
+      <c r="H86" s="43">
         <v>102.08</v>
       </c>
     </row>
     <row r="87" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B87" s="46" t="s">
+      <c r="B87" s="37" t="s">
         <v>119</v>
       </c>
       <c r="E87" s="28">
         <v>5</v>
       </c>
-      <c r="H87" s="37">
+      <c r="H87" s="43">
         <v>36.22</v>
       </c>
     </row>
     <row r="88" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B88" s="46" t="s">
+      <c r="B88" s="37" t="s">
         <v>120</v>
       </c>
-      <c r="H88" s="37">
+      <c r="H88" s="43">
         <v>27.96</v>
       </c>
     </row>
     <row r="89" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B89" s="46" t="s">
+      <c r="B89" s="37" t="s">
         <v>121</v>
       </c>
       <c r="E89" s="28">
         <v>10</v>
       </c>
-      <c r="H89" s="37">
+      <c r="H89" s="43">
         <v>34.450000000000003</v>
       </c>
     </row>
-    <row r="90" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B90" s="46" t="s">
+    <row r="90" spans="2:8" ht="27" x14ac:dyDescent="0.3">
+      <c r="B90" s="37" t="s">
         <v>122</v>
       </c>
       <c r="E90" s="28">
         <v>1</v>
       </c>
-      <c r="H90" s="37">
+      <c r="H90" s="43">
         <v>5.09</v>
       </c>
     </row>
     <row r="91" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B91" s="46" t="s">
+      <c r="B91" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="H91" s="37">
+      <c r="H91" s="43">
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="92" spans="2:8" ht="78" x14ac:dyDescent="0.3">
-      <c r="B92" s="46" t="s">
+    <row r="92" spans="2:8" ht="65.25" x14ac:dyDescent="0.3">
+      <c r="B92" s="37" t="s">
         <v>124</v>
       </c>
       <c r="E92" s="28">
         <v>9</v>
       </c>
-      <c r="H92" s="37">
+      <c r="H92" s="43">
         <v>33.79</v>
       </c>
     </row>
     <row r="93" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B93" s="46" t="s">
+      <c r="B93" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="H93" s="37">
+      <c r="H93" s="43">
         <v>27.96</v>
       </c>
     </row>
     <row r="94" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B94" s="46" t="s">
+      <c r="B94" s="37" t="s">
         <v>126</v>
       </c>
       <c r="E94" s="28">
         <v>5</v>
       </c>
-      <c r="H94" s="37">
+      <c r="H94" s="43">
         <v>25.66</v>
       </c>
     </row>
     <row r="95" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B95" s="46" t="s">
+      <c r="B95" s="37" t="s">
         <v>127</v>
       </c>
       <c r="E95" s="28">
         <v>4</v>
       </c>
-      <c r="H95" s="38">
+      <c r="H95" s="46">
         <v>34.700000000000003</v>
       </c>
     </row>
     <row r="96" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B96" s="46" t="s">
+      <c r="B96" s="37" t="s">
         <v>128</v>
       </c>
       <c r="E96" s="28">
         <v>10</v>
       </c>
-      <c r="H96" s="49">
+      <c r="H96" s="47">
         <v>165</v>
       </c>
     </row>
     <row r="97" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B97" s="46" t="s">
+      <c r="B97" s="37" t="s">
         <v>128</v>
       </c>
       <c r="E97" s="28">
         <v>15</v>
       </c>
-      <c r="H97" s="39">
+      <c r="H97" s="42">
         <v>12.32</v>
       </c>
     </row>
     <row r="98" spans="2:8" ht="103.5" x14ac:dyDescent="0.3">
-      <c r="B98" s="46" t="s">
+      <c r="B98" s="37" t="s">
         <v>129</v>
       </c>
       <c r="E98" s="28">
         <v>10</v>
       </c>
-      <c r="H98" s="39">
+      <c r="H98" s="42">
         <v>11.37</v>
       </c>
     </row>
     <row r="99" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B99" s="46" t="s">
+      <c r="B99" s="37" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="100" spans="2:8" ht="102" x14ac:dyDescent="0.3">
-      <c r="B100" s="47" t="s">
+    <row r="100" spans="2:8" ht="89.25" x14ac:dyDescent="0.3">
+      <c r="B100" s="38" t="s">
         <v>131</v>
       </c>
       <c r="E100" s="28">
@@ -2479,26 +2506,82 @@
         <v>12</v>
       </c>
     </row>
-    <row r="101" spans="2:8" ht="102" x14ac:dyDescent="0.3">
-      <c r="B101" s="47" t="s">
+    <row r="101" spans="2:8" ht="89.25" x14ac:dyDescent="0.3">
+      <c r="B101" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="E101" s="28">
-        <v>4</v>
+      <c r="E101" s="28" t="s">
+        <v>135</v>
       </c>
       <c r="F101" s="23">
+        <v>17</v>
+      </c>
+      <c r="H101" s="45">
         <v>34</v>
       </c>
     </row>
     <row r="102" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B102" s="40" t="s">
+      <c r="B102" s="31" t="s">
         <v>133</v>
       </c>
       <c r="F102" s="23">
         <v>6</v>
       </c>
-      <c r="H102" s="50">
+      <c r="H102" s="48">
         <v>207.26</v>
+      </c>
+    </row>
+    <row r="103" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B103" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="E103" s="28">
+        <v>12</v>
+      </c>
+      <c r="F103" s="23">
+        <v>10</v>
+      </c>
+      <c r="H103" s="45">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="104" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B104" s="31" t="s">
+        <v>136</v>
+      </c>
+      <c r="E104" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="F104" s="50">
+        <v>11.99</v>
+      </c>
+      <c r="H104" s="45">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="105" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B105" s="31" t="s">
+        <v>138</v>
+      </c>
+      <c r="E105" s="28">
+        <v>20</v>
+      </c>
+      <c r="H105" s="42">
+        <v>11.99</v>
+      </c>
+    </row>
+    <row r="106" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B106" s="31" t="s">
+        <v>139</v>
+      </c>
+      <c r="E106" s="28" t="s">
+        <v>140</v>
+      </c>
+      <c r="F106" s="23">
+        <v>11</v>
+      </c>
+      <c r="H106" s="45">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update tracker, expenses, settings, and misc assets
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cameroon_Shop_Purchase_Tracker.xlsx
+++ b/Cameroon_Shop_Purchase_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\cameroon-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42CF9A79-B8ED-4FA2-8370-C19FB7EACCAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7820BC2B-4212-4987-9D3E-A8076FB96D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-2616" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27420" yWindow="4005" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Americanselect shop tracker" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="146">
   <si>
     <t>TOTAL PURCHASE COST</t>
   </si>
@@ -457,6 +457,21 @@
   </si>
   <si>
     <t>10(5)</t>
+  </si>
+  <si>
+    <t>Oz Rechargeable Portable Blender Cup, Electric USB Juicer Blender, Mini Blender Portable Blender for Shakes And Smoothies, Juice</t>
+  </si>
+  <si>
+    <t>TG192 A Large Capacity 2400mAh Outdoor Wireless Speaker,</t>
+  </si>
+  <si>
+    <t>Men'S Electric Shaver</t>
+  </si>
+  <si>
+    <t>Digital Bathroom Scale, Electronic</t>
+  </si>
+  <si>
+    <t>Manual chopper</t>
   </si>
 </sst>
 </file>
@@ -467,7 +482,7 @@
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -545,43 +560,50 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF333333"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF222222"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF222222"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color rgb="FF2C3E50"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="14"/>
       <color rgb="FF0F1111"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="14"/>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -637,7 +659,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -693,30 +715,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="8" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -736,9 +734,39 @@
     <xf numFmtId="6" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="8" fontId="15" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="8" fontId="18" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="8" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="8" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1041,17 +1069,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.140625" customWidth="1"/>
-    <col min="2" max="2" width="23.42578125" style="31" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" style="43" customWidth="1"/>
     <col min="3" max="3" width="25.85546875" customWidth="1"/>
     <col min="4" max="4" width="22.42578125" style="2" customWidth="1"/>
     <col min="5" max="5" width="11.42578125" style="28" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" style="22" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.28515625" customWidth="1"/>
-    <col min="8" max="8" width="24.85546875" style="39" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" style="31" customWidth="1"/>
     <col min="9" max="9" width="18.42578125" customWidth="1"/>
     <col min="10" max="10" width="25" customWidth="1"/>
   </cols>
@@ -1060,9 +1088,9 @@
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31">
+      <c r="B1" s="43">
         <f>SUM(F:F)</f>
-        <v>303.89999999999998</v>
+        <v>321.02</v>
       </c>
       <c r="C1" s="8"/>
       <c r="D1" s="9"/>
@@ -1078,7 +1106,7 @@
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="31">
+      <c r="B2" s="43">
         <f>SUM(G:G)</f>
         <v>77.8</v>
       </c>
@@ -1096,9 +1124,9 @@
       <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="31">
+      <c r="B3" s="43">
         <f>SUM(H:H)</f>
-        <v>2386.9499999999998</v>
+        <v>2538.6999999999998</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="9"/>
@@ -1114,7 +1142,7 @@
       <c r="A4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="31">
+      <c r="B4" s="43">
         <f>SUM(K:K)</f>
         <v>0</v>
       </c>
@@ -1144,7 +1172,7 @@
       <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="43" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -1162,7 +1190,7 @@
       <c r="G6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="39" t="s">
+      <c r="H6" s="31" t="s">
         <v>11</v>
       </c>
       <c r="I6" s="8" t="s">
@@ -1178,11 +1206,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="44" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="8"/>
@@ -1207,9 +1235,9 @@
       </c>
       <c r="L7" s="8"/>
     </row>
-    <row r="8" spans="1:12" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A8" s="8"/>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="44" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="8"/>
@@ -1226,9 +1254,9 @@
       <c r="K8" s="8"/>
       <c r="L8" s="8"/>
     </row>
-    <row r="9" spans="1:12" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A9" s="8"/>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="44" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="8"/>
@@ -1245,9 +1273,9 @@
       <c r="K9" s="8"/>
       <c r="L9" s="8"/>
     </row>
-    <row r="10" spans="1:12" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="44" t="s">
         <v>20</v>
       </c>
       <c r="C10" s="8"/>
@@ -1264,9 +1292,9 @@
       <c r="K10" s="8"/>
       <c r="L10" s="8"/>
     </row>
-    <row r="11" spans="1:12" ht="27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A11" s="8"/>
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="44" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="8"/>
@@ -1283,9 +1311,9 @@
       <c r="K11" s="8"/>
       <c r="L11" s="8"/>
     </row>
-    <row r="12" spans="1:12" ht="27" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="44" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="8"/>
@@ -1302,9 +1330,9 @@
       <c r="K12" s="8"/>
       <c r="L12" s="8"/>
     </row>
-    <row r="13" spans="1:12" ht="27" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="56.25" x14ac:dyDescent="0.3">
       <c r="A13" s="8"/>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="44" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="8"/>
@@ -1321,9 +1349,9 @@
       <c r="K13" s="8"/>
       <c r="L13" s="8"/>
     </row>
-    <row r="14" spans="1:12" ht="27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="56.25" x14ac:dyDescent="0.3">
       <c r="A14" s="8"/>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="44" t="s">
         <v>24</v>
       </c>
       <c r="C14" s="8"/>
@@ -1340,9 +1368,9 @@
       <c r="K14" s="8"/>
       <c r="L14" s="8"/>
     </row>
-    <row r="15" spans="1:12" ht="27" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="44" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="8"/>
@@ -1359,9 +1387,9 @@
       <c r="K15" s="8"/>
       <c r="L15" s="8"/>
     </row>
-    <row r="16" spans="1:12" ht="27" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="56.25" x14ac:dyDescent="0.3">
       <c r="A16" s="8"/>
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="44" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="8"/>
@@ -1378,9 +1406,9 @@
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
     </row>
-    <row r="17" spans="1:12" ht="27" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="56.25" x14ac:dyDescent="0.3">
       <c r="A17" s="8"/>
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="44" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="8"/>
@@ -1397,9 +1425,9 @@
       <c r="K17" s="8"/>
       <c r="L17" s="8"/>
     </row>
-    <row r="18" spans="1:12" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A18" s="8"/>
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="44" t="s">
         <v>28</v>
       </c>
       <c r="C18" s="8"/>
@@ -1418,7 +1446,7 @@
     </row>
     <row r="19" spans="1:12" s="13" customFormat="1" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A19" s="16"/>
-      <c r="B19" s="31"/>
+      <c r="B19" s="43"/>
       <c r="C19" s="16"/>
       <c r="D19" s="17"/>
       <c r="E19" s="27"/>
@@ -1426,7 +1454,7 @@
       <c r="G19" s="18">
         <v>23.94</v>
       </c>
-      <c r="H19" s="40">
+      <c r="H19" s="32">
         <v>104.79</v>
       </c>
       <c r="I19" s="16"/>
@@ -1434,8 +1462,8 @@
       <c r="K19" s="16"/>
       <c r="L19" s="16"/>
     </row>
-    <row r="20" spans="1:12" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="32" t="s">
+    <row r="20" spans="1:12" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="44" t="s">
         <v>30</v>
       </c>
       <c r="D20" s="3" t="s">
@@ -1450,11 +1478,11 @@
       <c r="G20" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="H20" s="40">
+      <c r="H20" s="32">
         <v>69.73</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="28.5" x14ac:dyDescent="0.3">
       <c r="D21" s="3" t="s">
         <v>32</v>
       </c>
@@ -1467,13 +1495,13 @@
       <c r="G21" s="4">
         <v>32.799999999999997</v>
       </c>
-      <c r="H21" s="41"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H21" s="33"/>
+    </row>
+    <row r="22" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
         <v>46050</v>
       </c>
-      <c r="B22" s="31" t="s">
+      <c r="B22" s="43" t="s">
         <v>31</v>
       </c>
       <c r="D22" s="3"/>
@@ -1481,11 +1509,11 @@
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D23" s="3"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A24" s="5">
         <v>46053</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="43" t="s">
         <v>33</v>
       </c>
       <c r="C24" t="s">
@@ -1503,15 +1531,15 @@
       <c r="G24">
         <v>7.92</v>
       </c>
-      <c r="H24" s="42">
+      <c r="H24" s="34">
         <v>62.81</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="27" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="56.25" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
         <v>46053</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="43" t="s">
         <v>35</v>
       </c>
       <c r="C25" t="s">
@@ -1529,12 +1557,12 @@
       <c r="G25" s="4">
         <v>13.14</v>
       </c>
-      <c r="H25" s="42">
+      <c r="H25" s="34">
         <v>53.14</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="43" t="s">
         <v>37</v>
       </c>
       <c r="C26" t="s">
@@ -1549,12 +1577,12 @@
       <c r="F26" s="23">
         <v>8</v>
       </c>
-      <c r="H26" s="42">
+      <c r="H26" s="34">
         <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="43" t="s">
         <v>41</v>
       </c>
       <c r="C27" t="s">
@@ -1569,12 +1597,12 @@
       <c r="F27" s="22">
         <v>8</v>
       </c>
-      <c r="H27" s="42">
+      <c r="H27" s="34">
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B28" s="33" t="s">
+    <row r="28" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="B28" s="45" t="s">
         <v>43</v>
       </c>
       <c r="D28" s="2" t="s">
@@ -1586,12 +1614,12 @@
       <c r="F28" s="22">
         <v>10</v>
       </c>
-      <c r="H28" s="42">
+      <c r="H28" s="34">
         <v>34.89</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B29" s="33" t="s">
+    <row r="29" spans="1:12" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="B29" s="45" t="s">
         <v>45</v>
       </c>
       <c r="D29" s="2" t="s">
@@ -1603,12 +1631,12 @@
       <c r="F29" s="22">
         <v>10</v>
       </c>
-      <c r="H29" s="43">
+      <c r="H29" s="35">
         <v>34.86</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B30" s="33" t="s">
+    <row r="30" spans="1:12" ht="75" x14ac:dyDescent="0.3">
+      <c r="B30" s="45" t="s">
         <v>46</v>
       </c>
       <c r="D30" s="2" t="s">
@@ -1617,12 +1645,12 @@
       <c r="E30" s="28">
         <v>3</v>
       </c>
-      <c r="H30" s="43">
+      <c r="H30" s="35">
         <v>45.07</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="27" x14ac:dyDescent="0.3">
-      <c r="B31" s="33" t="s">
+    <row r="31" spans="1:12" ht="75" x14ac:dyDescent="0.3">
+      <c r="B31" s="45" t="s">
         <v>47</v>
       </c>
       <c r="D31" s="2" t="s">
@@ -1631,12 +1659,12 @@
       <c r="E31" s="28">
         <v>3</v>
       </c>
-      <c r="H31" s="43">
+      <c r="H31" s="35">
         <v>51.26</v>
       </c>
     </row>
-    <row r="32" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="33" t="s">
+    <row r="32" spans="1:12" s="6" customFormat="1" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="B32" s="45" t="s">
         <v>48</v>
       </c>
       <c r="D32" s="7" t="s">
@@ -1646,12 +1674,12 @@
         <v>1</v>
       </c>
       <c r="F32" s="22"/>
-      <c r="H32" s="43">
+      <c r="H32" s="35">
         <v>5.41</v>
       </c>
     </row>
-    <row r="33" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B33" s="33" t="s">
+    <row r="33" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B33" s="45" t="s">
         <v>49</v>
       </c>
       <c r="D33" s="7" t="s">
@@ -1660,12 +1688,12 @@
       <c r="E33" s="28">
         <v>3</v>
       </c>
-      <c r="H33" s="43">
+      <c r="H33" s="35">
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B34" s="33" t="s">
+    <row r="34" spans="2:8" ht="93.75" x14ac:dyDescent="0.3">
+      <c r="B34" s="45" t="s">
         <v>50</v>
       </c>
       <c r="D34" s="7" t="s">
@@ -1674,12 +1702,12 @@
       <c r="E34" s="28">
         <v>2</v>
       </c>
-      <c r="H34" s="43">
+      <c r="H34" s="35">
         <v>13.04</v>
       </c>
     </row>
-    <row r="35" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B35" s="33" t="s">
+    <row r="35" spans="2:8" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="B35" s="45" t="s">
         <v>51</v>
       </c>
       <c r="D35" s="7" t="s">
@@ -1688,12 +1716,12 @@
       <c r="E35" s="28">
         <v>2</v>
       </c>
-      <c r="H35" s="43">
+      <c r="H35" s="35">
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B36" s="33" t="s">
+    <row r="36" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B36" s="45" t="s">
         <v>52</v>
       </c>
       <c r="D36" s="7" t="s">
@@ -1702,12 +1730,12 @@
       <c r="E36" s="28">
         <v>2</v>
       </c>
-      <c r="H36" s="43">
+      <c r="H36" s="35">
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B37" s="33" t="s">
+    <row r="37" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B37" s="45" t="s">
         <v>53</v>
       </c>
       <c r="D37" s="7" t="s">
@@ -1716,12 +1744,12 @@
       <c r="E37" s="28">
         <v>1</v>
       </c>
-      <c r="H37" s="43">
+      <c r="H37" s="35">
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B38" s="33" t="s">
+    <row r="38" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B38" s="45" t="s">
         <v>54</v>
       </c>
       <c r="D38" s="7" t="s">
@@ -1730,12 +1758,12 @@
       <c r="E38" s="28">
         <v>10</v>
       </c>
-      <c r="H38" s="43">
+      <c r="H38" s="35">
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B39" s="33" t="s">
+    <row r="39" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B39" s="45" t="s">
         <v>55</v>
       </c>
       <c r="D39" s="7" t="s">
@@ -1744,12 +1772,12 @@
       <c r="E39" s="28">
         <v>1</v>
       </c>
-      <c r="H39" s="43">
+      <c r="H39" s="35">
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B40" s="33" t="s">
+    <row r="40" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B40" s="45" t="s">
         <v>56</v>
       </c>
       <c r="D40" s="7" t="s">
@@ -1758,12 +1786,12 @@
       <c r="E40" s="28">
         <v>1</v>
       </c>
-      <c r="H40" s="43">
+      <c r="H40" s="35">
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B41" s="33" t="s">
+    <row r="41" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B41" s="45" t="s">
         <v>57</v>
       </c>
       <c r="D41" s="7" t="s">
@@ -1772,12 +1800,12 @@
       <c r="E41" s="28">
         <v>1</v>
       </c>
-      <c r="H41" s="43">
+      <c r="H41" s="35">
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B42" s="33" t="s">
+    <row r="42" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B42" s="45" t="s">
         <v>58</v>
       </c>
       <c r="D42" s="7" t="s">
@@ -1786,12 +1814,12 @@
       <c r="E42" s="28">
         <v>1</v>
       </c>
-      <c r="H42" s="43">
+      <c r="H42" s="35">
         <v>12</v>
       </c>
     </row>
-    <row r="43" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B43" s="33" t="s">
+    <row r="43" spans="2:8" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="B43" s="45" t="s">
         <v>59</v>
       </c>
       <c r="D43" s="7" t="s">
@@ -1800,12 +1828,12 @@
       <c r="E43" s="28">
         <v>2</v>
       </c>
-      <c r="H43" s="43">
+      <c r="H43" s="35">
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B44" s="33" t="s">
+    <row r="44" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B44" s="45" t="s">
         <v>60</v>
       </c>
       <c r="D44" s="7" t="s">
@@ -1814,12 +1842,12 @@
       <c r="E44" s="28">
         <v>5</v>
       </c>
-      <c r="H44" s="43">
+      <c r="H44" s="35">
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B45" s="33" t="s">
+    <row r="45" spans="2:8" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="B45" s="45" t="s">
         <v>61</v>
       </c>
       <c r="D45" s="7" t="s">
@@ -1828,12 +1856,12 @@
       <c r="E45" s="28">
         <v>1</v>
       </c>
-      <c r="H45" s="43">
+      <c r="H45" s="35">
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B46" s="33" t="s">
+    <row r="46" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B46" s="45" t="s">
         <v>62</v>
       </c>
       <c r="D46" s="7" t="s">
@@ -1842,12 +1870,12 @@
       <c r="E46" s="28">
         <v>2</v>
       </c>
-      <c r="H46" s="43">
+      <c r="H46" s="35">
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B47" s="33" t="s">
+    <row r="47" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B47" s="45" t="s">
         <v>63</v>
       </c>
       <c r="D47" s="7" t="s">
@@ -1856,12 +1884,12 @@
       <c r="E47" s="28">
         <v>2</v>
       </c>
-      <c r="H47" s="43">
+      <c r="H47" s="35">
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B48" s="33" t="s">
+    <row r="48" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B48" s="45" t="s">
         <v>64</v>
       </c>
       <c r="D48" s="7" t="s">
@@ -1870,12 +1898,12 @@
       <c r="E48" s="28">
         <v>1</v>
       </c>
-      <c r="H48" s="43">
+      <c r="H48" s="35">
         <v>12</v>
       </c>
     </row>
-    <row r="49" spans="2:8" ht="89.25" x14ac:dyDescent="0.3">
-      <c r="B49" s="36" t="s">
+    <row r="49" spans="2:8" ht="206.25" x14ac:dyDescent="0.3">
+      <c r="B49" s="46" t="s">
         <v>65</v>
       </c>
       <c r="D49" s="7" t="s">
@@ -1884,12 +1912,12 @@
       <c r="E49" s="28">
         <v>1</v>
       </c>
-      <c r="H49" s="39">
+      <c r="H49" s="31">
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="2:8" ht="38.25" x14ac:dyDescent="0.3">
-      <c r="B50" s="36" t="s">
+    <row r="50" spans="2:8" ht="93.75" x14ac:dyDescent="0.3">
+      <c r="B50" s="46" t="s">
         <v>66</v>
       </c>
       <c r="D50" s="7" t="s">
@@ -1898,20 +1926,20 @@
       <c r="E50" s="28">
         <v>1</v>
       </c>
-      <c r="H50" s="39">
+      <c r="H50" s="31">
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B52" s="32" t="s">
+    <row r="52" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B52" s="44" t="s">
         <v>67</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="53" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B53" s="34" t="s">
+    <row r="53" spans="2:8" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="B53" s="47" t="s">
         <v>68</v>
       </c>
       <c r="C53" s="11" t="s">
@@ -1924,12 +1952,12 @@
       <c r="F53" s="24">
         <v>5.95</v>
       </c>
-      <c r="H53" s="44" t="s">
+      <c r="H53" s="36" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="54" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B54" s="34" t="s">
+    <row r="54" spans="2:8" ht="150" x14ac:dyDescent="0.25">
+      <c r="B54" s="47" t="s">
         <v>71</v>
       </c>
       <c r="C54" s="11" t="s">
@@ -1942,12 +1970,12 @@
       <c r="F54" s="24">
         <v>5.95</v>
       </c>
-      <c r="H54" s="44" t="s">
+      <c r="H54" s="36" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="55" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B55" s="34" t="s">
+    <row r="55" spans="2:8" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="B55" s="47" t="s">
         <v>73</v>
       </c>
       <c r="C55" s="11" t="s">
@@ -1960,12 +1988,12 @@
       <c r="F55" s="24">
         <v>5.95</v>
       </c>
-      <c r="H55" s="44" t="s">
+      <c r="H55" s="36" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="56" spans="2:8" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="B56" s="34" t="s">
+    <row r="56" spans="2:8" ht="131.25" x14ac:dyDescent="0.25">
+      <c r="B56" s="47" t="s">
         <v>75</v>
       </c>
       <c r="C56" s="11" t="s">
@@ -1978,12 +2006,12 @@
       <c r="F56" s="24">
         <v>5.95</v>
       </c>
-      <c r="H56" s="44" t="s">
+      <c r="H56" s="36" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="57" spans="2:8" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B57" s="34" t="s">
+    <row r="57" spans="2:8" ht="93.75" x14ac:dyDescent="0.25">
+      <c r="B57" s="47" t="s">
         <v>77</v>
       </c>
       <c r="C57" s="11" t="s">
@@ -1996,12 +2024,12 @@
       <c r="F57" s="24">
         <v>8.5</v>
       </c>
-      <c r="H57" s="44" t="s">
+      <c r="H57" s="36" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="58" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B58" s="34" t="s">
+    <row r="58" spans="2:8" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="B58" s="47" t="s">
         <v>80</v>
       </c>
       <c r="C58" s="11" t="s">
@@ -2014,12 +2042,12 @@
       <c r="F58" s="24">
         <v>5.5</v>
       </c>
-      <c r="H58" s="44" t="s">
+      <c r="H58" s="36" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="59" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B59" s="34" t="s">
+    <row r="59" spans="2:8" ht="131.25" x14ac:dyDescent="0.25">
+      <c r="B59" s="47" t="s">
         <v>83</v>
       </c>
       <c r="C59" s="11" t="s">
@@ -2032,12 +2060,12 @@
       <c r="F59" s="24">
         <v>5.95</v>
       </c>
-      <c r="H59" s="44" t="s">
+      <c r="H59" s="36" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="2:8" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B60" s="34" t="s">
+    <row r="60" spans="2:8" ht="93.75" x14ac:dyDescent="0.25">
+      <c r="B60" s="47" t="s">
         <v>85</v>
       </c>
       <c r="C60" s="11" t="s">
@@ -2050,12 +2078,12 @@
       <c r="F60" s="24">
         <v>5.5</v>
       </c>
-      <c r="H60" s="44" t="s">
+      <c r="H60" s="36" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="61" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B61" s="34" t="s">
+    <row r="61" spans="2:8" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="B61" s="47" t="s">
         <v>87</v>
       </c>
       <c r="C61" s="11" t="s">
@@ -2068,12 +2096,12 @@
       <c r="F61" s="24">
         <v>5.5</v>
       </c>
-      <c r="H61" s="44" t="s">
+      <c r="H61" s="36" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="62" spans="2:8" ht="51" x14ac:dyDescent="0.25">
-      <c r="B62" s="34" t="s">
+    <row r="62" spans="2:8" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="B62" s="47" t="s">
         <v>89</v>
       </c>
       <c r="C62" s="11" t="s">
@@ -2086,24 +2114,24 @@
       <c r="F62" s="24">
         <v>5.75</v>
       </c>
-      <c r="H62" s="44" t="s">
+      <c r="H62" s="36" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="63" spans="2:8" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="31"/>
+      <c r="B63" s="43"/>
       <c r="D63" s="14"/>
       <c r="E63" s="28"/>
       <c r="F63" s="22"/>
       <c r="G63" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="H63" s="44" t="s">
+      <c r="H63" s="36" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="64" spans="2:8" ht="51.75" x14ac:dyDescent="0.25">
-      <c r="B64" s="35" t="s">
+    <row r="64" spans="2:8" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="B64" s="48" t="s">
         <v>96</v>
       </c>
       <c r="E64" s="30">
@@ -2112,105 +2140,105 @@
       <c r="F64" s="25">
         <v>19.989999999999998</v>
       </c>
-      <c r="H64" s="41"/>
-    </row>
-    <row r="65" spans="2:11" ht="64.5" x14ac:dyDescent="0.25">
-      <c r="B65" s="35" t="s">
+      <c r="H64" s="33"/>
+    </row>
+    <row r="65" spans="2:11" ht="131.25" x14ac:dyDescent="0.3">
+      <c r="B65" s="48" t="s">
         <v>97</v>
       </c>
       <c r="E65" s="30">
         <v>3</v>
       </c>
       <c r="F65" s="26"/>
-      <c r="H65" s="49">
+      <c r="H65" s="41">
         <v>14.17</v>
       </c>
     </row>
-    <row r="66" spans="2:11" ht="90" x14ac:dyDescent="0.25">
-      <c r="B66" s="35" t="s">
+    <row r="66" spans="2:11" ht="206.25" x14ac:dyDescent="0.3">
+      <c r="B66" s="48" t="s">
         <v>98</v>
       </c>
       <c r="E66" s="30">
         <v>2</v>
       </c>
       <c r="F66" s="26"/>
-      <c r="H66" s="49">
+      <c r="H66" s="41">
         <v>23.99</v>
       </c>
     </row>
-    <row r="67" spans="2:11" ht="51.75" x14ac:dyDescent="0.25">
-      <c r="B67" s="35" t="s">
+    <row r="67" spans="2:11" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="B67" s="48" t="s">
         <v>99</v>
       </c>
       <c r="E67" s="30">
         <v>4</v>
       </c>
       <c r="F67" s="26"/>
-      <c r="H67" s="49">
+      <c r="H67" s="41">
         <v>21.98</v>
       </c>
     </row>
-    <row r="68" spans="2:11" ht="77.25" x14ac:dyDescent="0.25">
-      <c r="B68" s="35" t="s">
+    <row r="68" spans="2:11" ht="187.5" x14ac:dyDescent="0.3">
+      <c r="B68" s="48" t="s">
         <v>100</v>
       </c>
       <c r="E68" s="30">
         <v>3</v>
       </c>
       <c r="F68" s="26"/>
-      <c r="H68" s="49">
+      <c r="H68" s="41">
         <v>35.99</v>
       </c>
     </row>
-    <row r="69" spans="2:11" ht="77.25" x14ac:dyDescent="0.25">
-      <c r="B69" s="35" t="s">
+    <row r="69" spans="2:11" ht="150" x14ac:dyDescent="0.3">
+      <c r="B69" s="48" t="s">
         <v>101</v>
       </c>
       <c r="E69" s="30">
         <v>4</v>
       </c>
       <c r="F69" s="26"/>
-      <c r="H69" s="49">
+      <c r="H69" s="41">
         <v>22.76</v>
       </c>
     </row>
-    <row r="70" spans="2:11" ht="51.75" x14ac:dyDescent="0.25">
-      <c r="B70" s="35" t="s">
+    <row r="70" spans="2:11" ht="93.75" x14ac:dyDescent="0.3">
+      <c r="B70" s="48" t="s">
         <v>102</v>
       </c>
       <c r="E70" s="30">
         <v>4</v>
       </c>
       <c r="F70" s="26"/>
-      <c r="H70" s="49">
+      <c r="H70" s="41">
         <v>23.48</v>
       </c>
     </row>
-    <row r="71" spans="2:11" ht="51.75" x14ac:dyDescent="0.25">
-      <c r="B71" s="35" t="s">
+    <row r="71" spans="2:11" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="B71" s="48" t="s">
         <v>106</v>
       </c>
       <c r="E71" s="30">
         <v>4</v>
       </c>
       <c r="F71" s="26"/>
-      <c r="H71" s="49">
+      <c r="H71" s="41">
         <v>22.27</v>
       </c>
     </row>
-    <row r="72" spans="2:11" ht="27" x14ac:dyDescent="0.3">
-      <c r="B72" s="37" t="s">
+    <row r="72" spans="2:11" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B72" s="49" t="s">
         <v>107</v>
       </c>
       <c r="E72" s="30">
         <v>6</v>
       </c>
-      <c r="H72" s="42">
+      <c r="H72" s="34">
         <v>38.26</v>
       </c>
     </row>
-    <row r="73" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B73" s="37" t="s">
+    <row r="73" spans="2:11" ht="75" x14ac:dyDescent="0.3">
+      <c r="B73" s="49" t="s">
         <v>108</v>
       </c>
       <c r="E73" s="30">
@@ -2219,64 +2247,64 @@
       <c r="F73" s="23">
         <v>6</v>
       </c>
-      <c r="H73" s="42">
+      <c r="H73" s="34">
         <v>15.65</v>
       </c>
     </row>
-    <row r="74" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B74" s="37" t="s">
+    <row r="74" spans="2:11" ht="93.75" x14ac:dyDescent="0.3">
+      <c r="B74" s="49" t="s">
         <v>109</v>
       </c>
       <c r="E74" s="30">
         <v>4</v>
       </c>
-      <c r="H74" s="42">
+      <c r="H74" s="34">
         <v>20.11</v>
       </c>
     </row>
-    <row r="75" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B75" s="37" t="s">
+    <row r="75" spans="2:11" ht="75" x14ac:dyDescent="0.3">
+      <c r="B75" s="49" t="s">
         <v>110</v>
       </c>
       <c r="E75" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B76" s="37" t="s">
+    <row r="76" spans="2:11" ht="93.75" x14ac:dyDescent="0.3">
+      <c r="B76" s="49" t="s">
         <v>111</v>
       </c>
       <c r="E76" s="28">
         <v>15</v>
       </c>
-      <c r="H76" s="42">
+      <c r="H76" s="34">
         <v>31.5</v>
       </c>
     </row>
-    <row r="77" spans="2:11" ht="27" x14ac:dyDescent="0.3">
-      <c r="B77" s="37" t="s">
+    <row r="77" spans="2:11" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B77" s="49" t="s">
         <v>130</v>
       </c>
       <c r="E77" s="28">
         <v>6</v>
       </c>
-      <c r="H77" s="42">
+      <c r="H77" s="34">
         <v>23</v>
       </c>
     </row>
-    <row r="78" spans="2:11" ht="27" x14ac:dyDescent="0.3">
-      <c r="B78" s="37" t="s">
+    <row r="78" spans="2:11" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="B78" s="49" t="s">
         <v>112</v>
       </c>
       <c r="E78" s="28">
         <v>1</v>
       </c>
-      <c r="H78" s="42">
+      <c r="H78" s="34">
         <v>10.34</v>
       </c>
     </row>
-    <row r="79" spans="2:11" ht="27" x14ac:dyDescent="0.3">
-      <c r="B79" s="37" t="s">
+    <row r="79" spans="2:11" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B79" s="49" t="s">
         <v>113</v>
       </c>
       <c r="E79" s="28">
@@ -2285,21 +2313,21 @@
       <c r="F79" s="22">
         <v>3.68</v>
       </c>
-      <c r="H79" s="45">
+      <c r="H79" s="37">
         <v>23</v>
       </c>
     </row>
-    <row r="80" spans="2:11" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B80" s="37" t="s">
+    <row r="80" spans="2:11" ht="75" x14ac:dyDescent="0.3">
+      <c r="B80" s="49" t="s">
         <v>114</v>
       </c>
-      <c r="H80" s="42">
+      <c r="H80" s="34">
         <v>16</v>
       </c>
       <c r="K80" s="13"/>
     </row>
-    <row r="81" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B81" s="37" t="s">
+    <row r="81" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B81" s="49" t="s">
         <v>57</v>
       </c>
       <c r="E81" s="28">
@@ -2308,53 +2336,53 @@
       <c r="F81" s="22">
         <v>14</v>
       </c>
-      <c r="H81" s="45">
+      <c r="H81" s="37">
         <v>120</v>
       </c>
     </row>
-    <row r="82" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B82" s="37" t="s">
+    <row r="82" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B82" s="49" t="s">
         <v>115</v>
       </c>
-      <c r="H82" s="45">
+      <c r="H82" s="37">
         <v>75</v>
       </c>
     </row>
-    <row r="83" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B83" s="37" t="s">
+    <row r="83" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B83" s="49" t="s">
         <v>116</v>
       </c>
       <c r="E83" s="28">
         <v>2</v>
       </c>
-      <c r="H83" s="45">
+      <c r="H83" s="37">
         <v>10</v>
       </c>
     </row>
-    <row r="84" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B84" s="37" t="s">
+    <row r="84" spans="2:8" ht="93.75" x14ac:dyDescent="0.3">
+      <c r="B84" s="49" t="s">
         <v>117</v>
       </c>
       <c r="E84" s="28">
         <v>4</v>
       </c>
-      <c r="H84" s="45">
+      <c r="H84" s="37">
         <v>40</v>
       </c>
     </row>
-    <row r="85" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B85" s="37" t="s">
+    <row r="85" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B85" s="49" t="s">
         <v>118</v>
       </c>
       <c r="E85" s="28">
         <v>20</v>
       </c>
-      <c r="H85" s="45">
+      <c r="H85" s="37">
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B86" s="37" t="s">
+    <row r="86" spans="2:8" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="B86" s="49" t="s">
         <v>59</v>
       </c>
       <c r="E86" s="28">
@@ -2363,140 +2391,140 @@
       <c r="F86" s="22">
         <v>10.6</v>
       </c>
-      <c r="H86" s="43">
+      <c r="H86" s="35">
         <v>102.08</v>
       </c>
     </row>
-    <row r="87" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B87" s="37" t="s">
+    <row r="87" spans="2:8" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="B87" s="49" t="s">
         <v>119</v>
       </c>
       <c r="E87" s="28">
         <v>5</v>
       </c>
-      <c r="H87" s="43">
+      <c r="H87" s="35">
         <v>36.22</v>
       </c>
     </row>
-    <row r="88" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B88" s="37" t="s">
+    <row r="88" spans="2:8" ht="93.75" x14ac:dyDescent="0.3">
+      <c r="B88" s="49" t="s">
         <v>120</v>
       </c>
-      <c r="H88" s="43">
+      <c r="H88" s="35">
         <v>27.96</v>
       </c>
     </row>
-    <row r="89" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B89" s="37" t="s">
+    <row r="89" spans="2:8" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="B89" s="49" t="s">
         <v>121</v>
       </c>
       <c r="E89" s="28">
         <v>10</v>
       </c>
-      <c r="H89" s="43">
+      <c r="H89" s="35">
         <v>34.450000000000003</v>
       </c>
     </row>
-    <row r="90" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B90" s="37" t="s">
+    <row r="90" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B90" s="49" t="s">
         <v>122</v>
       </c>
       <c r="E90" s="28">
         <v>1</v>
       </c>
-      <c r="H90" s="43">
+      <c r="H90" s="35">
         <v>5.09</v>
       </c>
     </row>
-    <row r="91" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B91" s="37" t="s">
+    <row r="91" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B91" s="49" t="s">
         <v>123</v>
       </c>
-      <c r="H91" s="43">
+      <c r="H91" s="35">
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="92" spans="2:8" ht="65.25" x14ac:dyDescent="0.3">
-      <c r="B92" s="37" t="s">
+    <row r="92" spans="2:8" ht="150" x14ac:dyDescent="0.3">
+      <c r="B92" s="49" t="s">
         <v>124</v>
       </c>
       <c r="E92" s="28">
         <v>9</v>
       </c>
-      <c r="H92" s="43">
+      <c r="H92" s="35">
         <v>33.79</v>
       </c>
     </row>
-    <row r="93" spans="2:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="B93" s="37" t="s">
+    <row r="93" spans="2:8" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="B93" s="49" t="s">
         <v>125</v>
       </c>
-      <c r="H93" s="43">
+      <c r="H93" s="35">
         <v>27.96</v>
       </c>
     </row>
-    <row r="94" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B94" s="37" t="s">
+    <row r="94" spans="2:8" ht="75" x14ac:dyDescent="0.3">
+      <c r="B94" s="49" t="s">
         <v>126</v>
       </c>
       <c r="E94" s="28">
         <v>5</v>
       </c>
-      <c r="H94" s="43">
+      <c r="H94" s="35">
         <v>25.66</v>
       </c>
     </row>
-    <row r="95" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B95" s="37" t="s">
+    <row r="95" spans="2:8" ht="93.75" x14ac:dyDescent="0.3">
+      <c r="B95" s="49" t="s">
         <v>127</v>
       </c>
       <c r="E95" s="28">
         <v>4</v>
       </c>
-      <c r="H95" s="46">
+      <c r="H95" s="38">
         <v>34.700000000000003</v>
       </c>
     </row>
-    <row r="96" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B96" s="37" t="s">
+    <row r="96" spans="2:8" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="B96" s="49" t="s">
         <v>128</v>
       </c>
       <c r="E96" s="28">
         <v>10</v>
       </c>
-      <c r="H96" s="47">
+      <c r="H96" s="39">
         <v>165</v>
       </c>
     </row>
-    <row r="97" spans="2:8" ht="52.5" x14ac:dyDescent="0.3">
-      <c r="B97" s="37" t="s">
+    <row r="97" spans="2:8" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="B97" s="49" t="s">
         <v>128</v>
       </c>
       <c r="E97" s="28">
         <v>15</v>
       </c>
-      <c r="H97" s="42">
+      <c r="H97" s="34">
         <v>12.32</v>
       </c>
     </row>
-    <row r="98" spans="2:8" ht="103.5" x14ac:dyDescent="0.3">
-      <c r="B98" s="37" t="s">
+    <row r="98" spans="2:8" ht="206.25" x14ac:dyDescent="0.3">
+      <c r="B98" s="49" t="s">
         <v>129</v>
       </c>
       <c r="E98" s="28">
         <v>10</v>
       </c>
-      <c r="H98" s="42">
+      <c r="H98" s="34">
         <v>11.37</v>
       </c>
     </row>
-    <row r="99" spans="2:8" ht="39.75" x14ac:dyDescent="0.3">
-      <c r="B99" s="37" t="s">
+    <row r="99" spans="2:8" ht="93.75" x14ac:dyDescent="0.3">
+      <c r="B99" s="49" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="100" spans="2:8" ht="89.25" x14ac:dyDescent="0.3">
-      <c r="B100" s="38" t="s">
+    <row r="100" spans="2:8" ht="187.5" x14ac:dyDescent="0.3">
+      <c r="B100" s="50" t="s">
         <v>131</v>
       </c>
       <c r="E100" s="28">
@@ -2506,8 +2534,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="101" spans="2:8" ht="89.25" x14ac:dyDescent="0.3">
-      <c r="B101" s="38" t="s">
+    <row r="101" spans="2:8" ht="206.25" x14ac:dyDescent="0.3">
+      <c r="B101" s="50" t="s">
         <v>132</v>
       </c>
       <c r="E101" s="28" t="s">
@@ -2516,23 +2544,23 @@
       <c r="F101" s="23">
         <v>17</v>
       </c>
-      <c r="H101" s="45">
+      <c r="H101" s="37">
         <v>34</v>
       </c>
     </row>
-    <row r="102" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B102" s="31" t="s">
+    <row r="102" spans="2:8" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="B102" s="43" t="s">
         <v>133</v>
       </c>
       <c r="F102" s="23">
         <v>6</v>
       </c>
-      <c r="H102" s="48">
+      <c r="H102" s="40">
         <v>207.26</v>
       </c>
     </row>
-    <row r="103" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B103" s="31" t="s">
+    <row r="103" spans="2:8" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="B103" s="43" t="s">
         <v>134</v>
       </c>
       <c r="E103" s="28">
@@ -2541,37 +2569,37 @@
       <c r="F103" s="23">
         <v>10</v>
       </c>
-      <c r="H103" s="45">
+      <c r="H103" s="37">
         <v>30</v>
       </c>
     </row>
     <row r="104" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B104" s="31" t="s">
+      <c r="B104" s="43" t="s">
         <v>136</v>
       </c>
       <c r="E104" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="F104" s="50">
+      <c r="F104" s="42">
         <v>11.99</v>
       </c>
-      <c r="H104" s="45">
+      <c r="H104" s="37">
         <v>36</v>
       </c>
     </row>
     <row r="105" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B105" s="31" t="s">
+      <c r="B105" s="43" t="s">
         <v>138</v>
       </c>
       <c r="E105" s="28">
         <v>20</v>
       </c>
-      <c r="H105" s="42">
+      <c r="H105" s="34">
         <v>11.99</v>
       </c>
     </row>
-    <row r="106" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B106" s="31" t="s">
+    <row r="106" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B106" s="43" t="s">
         <v>139</v>
       </c>
       <c r="E106" s="28" t="s">
@@ -2580,8 +2608,69 @@
       <c r="F106" s="23">
         <v>11</v>
       </c>
-      <c r="H106" s="45">
+      <c r="H106" s="37">
         <v>22</v>
+      </c>
+    </row>
+    <row r="107" spans="2:8" ht="106.5" x14ac:dyDescent="0.3">
+      <c r="B107" s="52" t="s">
+        <v>141</v>
+      </c>
+      <c r="E107" s="28">
+        <v>5</v>
+      </c>
+      <c r="F107" s="42">
+        <v>4.12</v>
+      </c>
+      <c r="H107" s="34">
+        <v>20.239999999999998</v>
+      </c>
+    </row>
+    <row r="108" spans="2:8" ht="61.5" x14ac:dyDescent="0.3">
+      <c r="B108" s="52" t="s">
+        <v>142</v>
+      </c>
+      <c r="E108" s="28">
+        <v>5</v>
+      </c>
+      <c r="F108" s="23">
+        <v>13</v>
+      </c>
+      <c r="H108" s="37">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="109" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B109" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="E109" s="28">
+        <v>3</v>
+      </c>
+      <c r="H109" s="53">
+        <v>34.75</v>
+      </c>
+    </row>
+    <row r="110" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B110" s="51" t="s">
+        <v>144</v>
+      </c>
+      <c r="E110" s="28">
+        <v>2</v>
+      </c>
+      <c r="H110" s="54">
+        <v>19.760000000000002</v>
+      </c>
+    </row>
+    <row r="111" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B111" s="43" t="s">
+        <v>145</v>
+      </c>
+      <c r="E111" s="28">
+        <v>2</v>
+      </c>
+      <c r="H111" s="37">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>